<commit_message>
Results for stopping criteria are updated
</commit_message>
<xml_diff>
--- a/SC reuslts/some results NSGAII.xlsx
+++ b/SC reuslts/some results NSGAII.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mahbub\Documents\GitHub\EnergyPLANDomainKnowledgeEAStep1\SC reuslts\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20730" windowHeight="11385" activeTab="7"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20730" windowHeight="11385"/>
   </bookViews>
   <sheets>
     <sheet name="ZDT1" sheetId="1" r:id="rId1"/>
@@ -20,7 +25,7 @@
     <externalReference r:id="rId9"/>
     <externalReference r:id="rId10"/>
   </externalReferences>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -110,8 +115,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -237,7 +242,17 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
   <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
   <c:chart>
     <c:title>
       <c:tx>
@@ -270,6 +285,7 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
         <a:ln>
@@ -278,10 +294,12 @@
         <a:effectLst/>
       </c:spPr>
     </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
         <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
@@ -1805,14 +1823,23 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="67547136"/>
-        <c:axId val="67549056"/>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="296246264"/>
+        <c:axId val="296246656"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="67547136"/>
+        <c:axId val="296246264"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
+        <c:delete val="0"/>
         <c:axPos val="b"/>
         <c:majorGridlines>
           <c:spPr>
@@ -1854,6 +1881,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
             <a:ln>
@@ -1863,6 +1891,7 @@
           </c:spPr>
         </c:title>
         <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
@@ -1894,18 +1923,19 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67549056"/>
+        <c:crossAx val="296246656"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="67549056"/>
+        <c:axId val="296246656"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
+        <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:majorGridlines>
           <c:spPr>
@@ -1947,6 +1977,7 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
             <a:ln>
@@ -1957,6 +1988,7 @@
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
@@ -1988,10 +2020,10 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="it-IT"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67547136"/>
+        <c:crossAx val="296246264"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2005,6 +2037,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2028,7 +2061,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="en-US"/>
+      <a:endParaRPr lang="it-IT"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -2341,6 +2374,87 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="TextBox 4"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6819900" y="3190875"/>
+          <a:ext cx="6486525" cy="1219200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>This files report the HVd,</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="it-IT" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> epsd, HVper, evaluation saves parameters for each problem (tabs) when comparing with 500 generations for NSGAII. The summary tab report the summarized view of all the parameters. Please note that this file is linked to "some results SPEA2.xlsx" file (in summary tab) to provided report for SPEA2. </a:t>
+          </a:r>
+          <a:endParaRPr lang="it-IT" sz="1100">
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -2731,7 +2845,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Sheet1"/>
@@ -5242,7 +5356,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="ZDT1"/>
@@ -6942,7 +7056,7 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="4"/>
       <sheetData sheetId="5">
         <row r="4">
           <cell r="C4">
@@ -8047,16 +8161,16 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:V34"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.28515625" customWidth="1"/>
@@ -8066,7 +8180,7 @@
     <col min="7" max="7" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -8080,7 +8194,7 @@
         <v>0.66616012487499998</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -8100,7 +8214,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>0</v>
       </c>
@@ -8120,7 +8234,7 @@
         <v>-8.1951611083141897E-4</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>1</v>
       </c>
@@ -8140,7 +8254,7 @@
         <v>-3.6281739877806699E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>2</v>
       </c>
@@ -8160,7 +8274,7 @@
         <v>4.5989107833585502E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>3</v>
       </c>
@@ -8180,7 +8294,7 @@
         <v>-4.6405229793171797E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>4</v>
       </c>
@@ -8200,7 +8314,7 @@
         <v>-1.0926191401774399E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>5</v>
       </c>
@@ -8220,7 +8334,7 @@
         <v>-3.8592048051273001E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>6</v>
       </c>
@@ -8240,7 +8354,7 @@
         <v>-5.2609140308685302E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>7</v>
       </c>
@@ -8260,7 +8374,7 @@
         <v>-3.4882202136190901E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>8</v>
       </c>
@@ -8280,7 +8394,7 @@
         <v>-3.7796113035970498E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>9</v>
       </c>
@@ -8300,7 +8414,7 @@
         <v>-2.3133702247160599E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10</v>
       </c>
@@ -8320,7 +8434,7 @@
         <v>-5.5167273454262899E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>11</v>
       </c>
@@ -8340,7 +8454,7 @@
         <v>-5.6387585042915103E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>12</v>
       </c>
@@ -8360,7 +8474,7 @@
         <v>1.5256660666840801E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:22">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>13</v>
       </c>
@@ -8380,7 +8494,7 @@
         <v>-6.9065711255477296E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:22">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>14</v>
       </c>
@@ -8424,7 +8538,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="19" spans="1:22">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>15</v>
       </c>
@@ -8448,7 +8562,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:22">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>16</v>
       </c>
@@ -8472,7 +8586,7 @@
         <v>37.5</v>
       </c>
     </row>
-    <row r="21" spans="1:22">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>17</v>
       </c>
@@ -8492,7 +8606,7 @@
         <v>-1.1920192462140201E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:22">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>18</v>
       </c>
@@ -8512,7 +8626,7 @@
         <v>-6.97531516784921E-4</v>
       </c>
     </row>
-    <row r="23" spans="1:22">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>19</v>
       </c>
@@ -8532,7 +8646,7 @@
         <v>1.5421856974445701E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:22">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>20</v>
       </c>
@@ -8552,7 +8666,7 @@
         <v>-3.16746410373868E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:22">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>21</v>
       </c>
@@ -8572,7 +8686,7 @@
         <v>-4.3057009789222401E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:22">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>22</v>
       </c>
@@ -8592,7 +8706,7 @@
         <v>-4.0151606948934902E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:22">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>23</v>
       </c>
@@ -8612,7 +8726,7 @@
         <v>-1.78892856657361E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:22">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>24</v>
       </c>
@@ -8632,7 +8746,7 @@
         <v>-6.8941063092096098E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:22">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>25</v>
       </c>
@@ -8652,7 +8766,7 @@
         <v>-7.5661382731223503E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:22">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>26</v>
       </c>
@@ -8672,7 +8786,7 @@
         <v>-5.39067138134274E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:22">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>27</v>
       </c>
@@ -8692,7 +8806,7 @@
         <v>1.8114772385106001E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:22">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>28</v>
       </c>
@@ -8712,7 +8826,7 @@
         <v>-1.11879807624626E-3</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>29</v>
       </c>
@@ -8732,7 +8846,7 @@
         <v>1.60627969693857E-3</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>8</v>
       </c>
@@ -8756,9 +8870,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G50"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -8768,7 +8882,7 @@
     <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -8782,7 +8896,7 @@
         <v>0.33283355941638099</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -8802,7 +8916,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0</v>
       </c>
@@ -8822,7 +8936,7 @@
         <v>-8.0974129452271405E-4</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -8842,7 +8956,7 @@
         <v>1.1177611943135001E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2</v>
       </c>
@@ -8862,7 +8976,7 @@
         <v>-3.2857375677534601E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>
@@ -8882,7 +8996,7 @@
         <v>-2.1183220238527498E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>4</v>
       </c>
@@ -8902,7 +9016,7 @@
         <v>-1.8999241952578599E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>5</v>
       </c>
@@ -8922,7 +9036,7 @@
         <v>1.9119309980650801E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>6</v>
       </c>
@@ -8942,7 +9056,7 @@
         <v>-7.0782432186709196E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>7</v>
       </c>
@@ -8962,7 +9076,7 @@
         <v>-2.0304782157437801E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>8</v>
       </c>
@@ -8982,7 +9096,7 @@
         <v>-2.4605847340881601E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>9</v>
       </c>
@@ -9002,7 +9116,7 @@
         <v>-4.0997083396021499E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10</v>
       </c>
@@ -9022,7 +9136,7 @@
         <v>-2.81743809917434E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>11</v>
       </c>
@@ -9042,7 +9156,7 @@
         <v>-5.5938596089526397E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>12</v>
       </c>
@@ -9062,7 +9176,7 @@
         <v>2.2675628621779899E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>13</v>
       </c>
@@ -9082,7 +9196,7 @@
         <v>-9.0659135082225796E-4</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>14</v>
       </c>
@@ -9102,7 +9216,7 @@
         <v>-4.5720977475325296E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>15</v>
       </c>
@@ -9122,7 +9236,7 @@
         <v>-2.7016668219681499E-3</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>16</v>
       </c>
@@ -9142,7 +9256,7 @@
         <v>-3.2667375157225901E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>17</v>
       </c>
@@ -9162,7 +9276,7 @@
         <v>5.8314486047872297E-5</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>18</v>
       </c>
@@ -9182,7 +9296,7 @@
         <v>-1.7238776689698599E-4</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>19</v>
       </c>
@@ -9202,7 +9316,7 @@
         <v>-9.5777867510127204E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>20</v>
       </c>
@@ -9222,7 +9336,7 @@
         <v>9.0615851833464301E-4</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>21</v>
       </c>
@@ -9242,7 +9356,7 @@
         <v>-5.4431932951686203E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>22</v>
       </c>
@@ -9262,7 +9376,7 @@
         <v>-3.5403511139828702E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>23</v>
       </c>
@@ -9282,7 +9396,7 @@
         <v>-3.6472321048567299E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>24</v>
       </c>
@@ -9302,7 +9416,7 @@
         <v>2.6832081451161299E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>25</v>
       </c>
@@ -9322,7 +9436,7 @@
         <v>-3.5274571843107999E-4</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>26</v>
       </c>
@@ -9342,7 +9456,7 @@
         <v>2.5990513066531602E-4</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>27</v>
       </c>
@@ -9362,7 +9476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>28</v>
       </c>
@@ -9382,7 +9496,7 @@
         <v>5.0382563890175496E-3</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>29</v>
       </c>
@@ -9402,7 +9516,7 @@
         <v>-1.60338391865949E-3</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>8</v>
       </c>
@@ -9418,7 +9532,7 @@
         <v>0.96701436612971825</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D39">
         <f>QUARTILE($D$4:$D$33,0)</f>
         <v>-2.7925113231100302E-3</v>
@@ -9432,7 +9546,7 @@
         <v>-7.0782432186709196E-3</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D40">
         <f>QUARTILE($D$4:$D$33,1)</f>
         <v>3.9509089179294387E-4</v>
@@ -9446,7 +9560,7 @@
         <v>-3.3493909543108125E-3</v>
       </c>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D41">
         <f>QUARTILE($D$4:$D$33,2)</f>
         <v>2.8199461243420499E-3</v>
@@ -9460,7 +9574,7 @@
         <v>-1.7516540569586748E-3</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D42">
         <f>QUARTILE($D$4:$D$33,3)</f>
         <v>4.2106787343501647E-3</v>
@@ -9474,7 +9588,7 @@
         <v>1.0871214720223323E-4</v>
       </c>
     </row>
-    <row r="43" spans="1:7">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D43">
         <f>QUARTILE($D$4:$D$33,4)</f>
         <v>6.3749054886274503E-3</v>
@@ -9488,7 +9602,7 @@
         <v>5.0382563890175496E-3</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D45">
         <f>D38-D37</f>
         <v>0</v>
@@ -9498,7 +9612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D46">
         <f>D39-D38</f>
         <v>-2.7925113231100302E-3</v>
@@ -9508,7 +9622,7 @@
         <v>7.0782432186709196E-3</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D47">
         <f t="shared" ref="D47:D50" si="0">D40-D39</f>
         <v>3.1876022149029742E-3</v>
@@ -9518,7 +9632,7 @@
         <v>-3.7288522643601071E-3</v>
       </c>
     </row>
-    <row r="48" spans="1:7">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D48">
         <f t="shared" si="0"/>
         <v>2.4248552325491059E-3</v>
@@ -9528,7 +9642,7 @@
         <v>-1.5977368973521377E-3</v>
       </c>
     </row>
-    <row r="49" spans="4:6">
+    <row r="49" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D49">
         <f t="shared" si="0"/>
         <v>1.3907326100081148E-3</v>
@@ -9538,7 +9652,7 @@
         <v>-1.860366204160908E-3</v>
       </c>
     </row>
-    <row r="50" spans="4:6">
+    <row r="50" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D50">
         <f t="shared" si="0"/>
         <v>2.1642267542772856E-3</v>
@@ -9555,9 +9669,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F50"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -9567,7 +9681,7 @@
     <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -9581,7 +9695,7 @@
         <v>0.51719187154758695</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -9601,7 +9715,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0</v>
       </c>
@@ -9621,7 +9735,7 @@
         <v>-1.2119754075568499E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -9641,7 +9755,7 @@
         <v>-5.9026780993743999E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2</v>
       </c>
@@ -9661,7 +9775,7 @@
         <v>1.31836055900639E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>
@@ -9681,7 +9795,7 @@
         <v>-1.67674038697403E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>4</v>
       </c>
@@ -9701,7 +9815,7 @@
         <v>-1.0142672573018E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>5</v>
       </c>
@@ -9721,7 +9835,7 @@
         <v>-1.2517411531936799E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>6</v>
       </c>
@@ -9741,7 +9855,7 @@
         <v>1.9154975424234199E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>7</v>
       </c>
@@ -9761,7 +9875,7 @@
         <v>-6.99970418727946E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>8</v>
       </c>
@@ -9781,7 +9895,7 @@
         <v>-3.2579873770000002E-4</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>9</v>
       </c>
@@ -9801,7 +9915,7 @@
         <v>-2.6419898658634998E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10</v>
       </c>
@@ -9821,7 +9935,7 @@
         <v>-1.3954769173487499E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>11</v>
       </c>
@@ -9841,7 +9955,7 @@
         <v>-4.8550550644500803E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>12</v>
       </c>
@@ -9861,7 +9975,7 @@
         <v>-5.0990232070927399E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>13</v>
       </c>
@@ -9881,7 +9995,7 @@
         <v>-1.7819612863766499E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>14</v>
       </c>
@@ -9901,7 +10015,7 @@
         <v>-1.1371158191845501E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>15</v>
       </c>
@@ -9921,7 +10035,7 @@
         <v>3.9224771035693801E-4</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>16</v>
       </c>
@@ -9941,7 +10055,7 @@
         <v>-1.3571533176202999E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>17</v>
       </c>
@@ -9961,7 +10075,7 @@
         <v>-2.6017640606640298E-4</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>18</v>
       </c>
@@ -9981,7 +10095,7 @@
         <v>-5.7224645484128204E-3</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>19</v>
       </c>
@@ -10001,7 +10115,7 @@
         <v>-8.8889988539172793E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>20</v>
       </c>
@@ -10021,7 +10135,7 @@
         <v>-5.8806215826587198E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>21</v>
       </c>
@@ -10041,7 +10155,7 @@
         <v>-2.59241435319469E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>22</v>
       </c>
@@ -10061,7 +10175,7 @@
         <v>-6.6292179250593501E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>23</v>
       </c>
@@ -10081,7 +10195,7 @@
         <v>-1.0078287593559099E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>24</v>
       </c>
@@ -10101,7 +10215,7 @@
         <v>-6.3987936206359999E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>25</v>
       </c>
@@ -10121,7 +10235,7 @@
         <v>-8.1884611163008502E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>26</v>
       </c>
@@ -10141,7 +10255,7 @@
         <v>-8.6311564224213905E-4</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>27</v>
       </c>
@@ -10161,7 +10275,7 @@
         <v>-8.2549595578293705E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>28</v>
       </c>
@@ -10181,7 +10295,7 @@
         <v>-1.08959930176485E-3</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>29</v>
       </c>
@@ -10201,7 +10315,7 @@
         <v>-7.0021476630840996E-4</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>8</v>
       </c>
@@ -10217,7 +10331,7 @@
         <v>0.98451978129199669</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D39">
         <f>QUARTILE($D$4:$D$33,0)</f>
         <v>-5.6410577857612899E-4</v>
@@ -10227,7 +10341,7 @@
         <v>-1.3954769173487499E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D40">
         <f>QUARTILE($D$4:$D$33,1)</f>
         <v>2.1502800157512875E-3</v>
@@ -10237,7 +10351,7 @@
         <v>-7.8912718840455018E-3</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D41">
         <f>QUARTILE($D$4:$D$33,2)</f>
         <v>4.4350223274996449E-3</v>
@@ -10247,7 +10361,7 @@
         <v>-4.9770391357714105E-3</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D42">
         <f>QUARTILE($D$4:$D$33,3)</f>
         <v>6.0704804641376602E-3</v>
@@ -10257,7 +10371,7 @@
         <v>-1.1201933282128499E-3</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D43">
         <f>QUARTILE($D$4:$D$33,4)</f>
         <v>1.06046338090119E-2</v>
@@ -10267,7 +10381,7 @@
         <v>1.9154975424234199E-3</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D45">
         <f>D38-D37</f>
         <v>0</v>
@@ -10277,7 +10391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D46">
         <f>D39-D38</f>
         <v>-5.6410577857612899E-4</v>
@@ -10287,7 +10401,7 @@
         <v>-1.3954769173487499E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D47">
         <f t="shared" ref="D47:F50" si="0">D40-D39</f>
         <v>2.7143857943274165E-3</v>
@@ -10297,7 +10411,7 @@
         <v>6.0634972894419974E-3</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D48">
         <f t="shared" si="0"/>
         <v>2.2847423117483574E-3</v>
@@ -10307,7 +10421,7 @@
         <v>2.9142327482740912E-3</v>
       </c>
     </row>
-    <row r="49" spans="4:6">
+    <row r="49" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D49">
         <f t="shared" si="0"/>
         <v>1.6354581366380154E-3</v>
@@ -10317,7 +10431,7 @@
         <v>3.8568458075585606E-3</v>
       </c>
     </row>
-    <row r="50" spans="4:6">
+    <row r="50" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D50">
         <f t="shared" si="0"/>
         <v>4.5341533448742394E-3</v>
@@ -10334,9 +10448,9 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F34"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -10346,7 +10460,7 @@
     <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -10360,7 +10474,7 @@
         <v>0.66617361728492197</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -10380,7 +10494,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0</v>
       </c>
@@ -10400,7 +10514,7 @@
         <v>4.0554145517913099E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -10420,7 +10534,7 @@
         <v>0.279595935073226</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2</v>
       </c>
@@ -10440,7 +10554,7 @@
         <v>-1.8706740924329099E-4</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>
@@ -10460,7 +10574,7 @@
         <v>-3.2570612161153501E-4</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>4</v>
       </c>
@@ -10480,7 +10594,7 @@
         <v>-0.25458930937267898</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>5</v>
       </c>
@@ -10500,7 +10614,7 @@
         <v>-0.21675477052320299</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>6</v>
       </c>
@@ -10520,7 +10634,7 @@
         <v>2.91664938337582E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>7</v>
       </c>
@@ -10540,7 +10654,7 @@
         <v>0.104297651062652</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>8</v>
       </c>
@@ -10560,7 +10674,7 @@
         <v>4.3715158959601796E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>9</v>
       </c>
@@ -10580,7 +10694,7 @@
         <v>-3.91949096680555E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10</v>
       </c>
@@ -10600,7 +10714,7 @@
         <v>1.91910487543472E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>11</v>
       </c>
@@ -10620,7 +10734,7 @@
         <v>-6.0679295346903099E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>12</v>
       </c>
@@ -10640,7 +10754,7 @@
         <v>3.9748435611588204E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>13</v>
       </c>
@@ -10660,7 +10774,7 @@
         <v>5.7916706645013598E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>14</v>
       </c>
@@ -10680,7 +10794,7 @@
         <v>4.2894481460590802E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>15</v>
       </c>
@@ -10700,7 +10814,7 @@
         <v>7.8711482512001205E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>16</v>
       </c>
@@ -10720,7 +10834,7 @@
         <v>1.4486254408815299E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>17</v>
       </c>
@@ -10740,7 +10854,7 @@
         <v>9.8627864801995702E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>18</v>
       </c>
@@ -10760,7 +10874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>19</v>
       </c>
@@ -10780,7 +10894,7 @@
         <v>-9.7910468117792998E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>20</v>
       </c>
@@ -10800,7 +10914,7 @@
         <v>4.7719312585747797E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>21</v>
       </c>
@@ -10820,7 +10934,7 @@
         <v>2.1047689339612698E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>22</v>
       </c>
@@ -10840,7 +10954,7 @@
         <v>-5.5136005584197002E-4</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>23</v>
       </c>
@@ -10860,7 +10974,7 @@
         <v>-7.6083237656365799E-4</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>24</v>
       </c>
@@ -10880,7 +10994,7 @@
         <v>5.2323261747570697E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>25</v>
       </c>
@@ -10900,7 +11014,7 @@
         <v>0.131960652140344</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>26</v>
       </c>
@@ -10920,7 +11034,7 @@
         <v>5.1836604315231599E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>27</v>
       </c>
@@ -10940,7 +11054,7 @@
         <v>-1.80039045323332E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>28</v>
       </c>
@@ -10960,7 +11074,7 @@
         <v>6.6104754297627803E-3</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>29</v>
       </c>
@@ -10980,7 +11094,7 @@
         <v>0.27240253349211102</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>8</v>
       </c>
@@ -11003,9 +11117,9 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F55"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -11015,7 +11129,7 @@
     <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -11029,7 +11143,7 @@
         <v>0.40590724234006298</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -11049,7 +11163,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0</v>
       </c>
@@ -11069,7 +11183,7 @@
         <v>3.8198108154760902E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -11089,7 +11203,7 @@
         <v>-1.2142214752381799</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2</v>
       </c>
@@ -11109,7 +11223,7 @@
         <v>-7.0074214958807002E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>
@@ -11129,7 +11243,7 @@
         <v>9.3640710508028097E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>4</v>
       </c>
@@ -11149,7 +11263,7 @@
         <v>-1.1840350230275001</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>5</v>
       </c>
@@ -11169,7 +11283,7 @@
         <v>-0.34271872271019399</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>6</v>
       </c>
@@ -11189,7 +11303,7 @@
         <v>1.54688456743761E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>7</v>
       </c>
@@ -11209,7 +11323,7 @@
         <v>-2.01434853155701E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>8</v>
       </c>
@@ -11229,7 +11343,7 @@
         <v>1.4505734973628399E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>9</v>
       </c>
@@ -11249,7 +11363,7 @@
         <v>8.9788680184770594E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10</v>
       </c>
@@ -11269,7 +11383,7 @@
         <v>1.5916220751723699E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>11</v>
       </c>
@@ -11289,7 +11403,7 @@
         <v>-0.31100727658218902</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>12</v>
       </c>
@@ -11309,7 +11423,7 @@
         <v>-5.0674695337909699E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>13</v>
       </c>
@@ -11329,7 +11443,7 @@
         <v>-8.5323927216879494E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>14</v>
       </c>
@@ -11349,7 +11463,7 @@
         <v>1.5645896908951299E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>15</v>
       </c>
@@ -11369,7 +11483,7 @@
         <v>-2.3754180001397399E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>16</v>
       </c>
@@ -11389,7 +11503,7 @@
         <v>-1.06692643429668</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>17</v>
       </c>
@@ -11409,7 +11523,7 @@
         <v>1.6243311531219599E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>18</v>
       </c>
@@ -11429,7 +11543,7 @@
         <v>-0.46301180079864301</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>19</v>
       </c>
@@ -11449,7 +11563,7 @@
         <v>-1.69854676244289</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>20</v>
       </c>
@@ -11469,7 +11583,7 @@
         <v>-0.94912546798061004</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>21</v>
       </c>
@@ -11489,7 +11603,7 @@
         <v>-1.80430025814446</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>22</v>
       </c>
@@ -11509,7 +11623,7 @@
         <v>1.33636024190034E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>23</v>
       </c>
@@ -11529,7 +11643,7 @@
         <v>-0.25131193831996201</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>24</v>
       </c>
@@ -11549,7 +11663,7 @@
         <v>-0.48756962261563502</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>25</v>
       </c>
@@ -11569,7 +11683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>26</v>
       </c>
@@ -11589,7 +11703,7 @@
         <v>-2.6095160997089502E-4</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>27</v>
       </c>
@@ -11609,7 +11723,7 @@
         <v>-0.74697105233851402</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>28</v>
       </c>
@@ -11629,7 +11743,7 @@
         <v>1.8625747914139301E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>29</v>
       </c>
@@ -11649,7 +11763,7 @@
         <v>-0.38463177904765999</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>8</v>
       </c>
@@ -11665,7 +11779,7 @@
         <v>0.57649171111802644</v>
       </c>
     </row>
-    <row r="55" spans="6:6">
+    <row r="55" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F55" s="1"/>
     </row>
   </sheetData>
@@ -11680,9 +11794,9 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F34"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -11692,7 +11806,7 @@
     <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -11706,7 +11820,7 @@
         <v>0.46783583650461702</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -11726,7 +11840,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0</v>
       </c>
@@ -11746,7 +11860,7 @@
         <v>-3.6535029671500102E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -11766,7 +11880,7 @@
         <v>1.4675506133468E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2</v>
       </c>
@@ -11786,7 +11900,7 @@
         <v>-2.3010561786476701E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>
@@ -11806,7 +11920,7 @@
         <v>-2.9082730606477199E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>4</v>
       </c>
@@ -11826,7 +11940,7 @@
         <v>3.3547020427374799E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>5</v>
       </c>
@@ -11846,7 +11960,7 @@
         <v>-2.7226830001258098E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>6</v>
       </c>
@@ -11866,7 +11980,7 @@
         <v>1.47153077308439E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>7</v>
       </c>
@@ -11886,7 +12000,7 @@
         <v>2.6752615165469101E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>8</v>
       </c>
@@ -11906,7 +12020,7 @@
         <v>4.3015006239444598E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>9</v>
       </c>
@@ -11926,7 +12040,7 @@
         <v>-1.2398493184265801E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10</v>
       </c>
@@ -11946,7 +12060,7 @@
         <v>-1.1238123454104E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>11</v>
       </c>
@@ -11966,7 +12080,7 @@
         <v>-6.4259516686617701E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>12</v>
       </c>
@@ -11986,7 +12100,7 @@
         <v>-1.5040684506399201E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>13</v>
       </c>
@@ -12006,7 +12120,7 @@
         <v>1.1710418563115599E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>14</v>
       </c>
@@ -12026,7 +12140,7 @@
         <v>-1.8614187586653699E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>15</v>
       </c>
@@ -12046,7 +12160,7 @@
         <v>-2.11779337502087E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>16</v>
       </c>
@@ -12066,7 +12180,7 @@
         <v>2.9152638894912502E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>17</v>
       </c>
@@ -12086,7 +12200,7 @@
         <v>9.1143764287142798E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>18</v>
       </c>
@@ -12106,7 +12220,7 @@
         <v>2.9163089003310799E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>19</v>
       </c>
@@ -12126,7 +12240,7 @@
         <v>-7.3466645591996305E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>20</v>
       </c>
@@ -12146,7 +12260,7 @@
         <v>-1.4474323063490099E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>21</v>
       </c>
@@ -12166,7 +12280,7 @@
         <v>-1.4666085283480399E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>22</v>
       </c>
@@ -12186,7 +12300,7 @@
         <v>5.4873279348653901E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>23</v>
       </c>
@@ -12206,7 +12320,7 @@
         <v>3.3292849450299498E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>24</v>
       </c>
@@ -12226,7 +12340,7 @@
         <v>1.8729859539121201E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>25</v>
       </c>
@@ -12246,7 +12360,7 @@
         <v>2.3295079612731802E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>26</v>
       </c>
@@ -12266,7 +12380,7 @@
         <v>-8.20997221326214E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>27</v>
       </c>
@@ -12286,7 +12400,7 @@
         <v>7.7431777921155298E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>28</v>
       </c>
@@ -12306,7 +12420,7 @@
         <v>3.8305146468709902E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>29</v>
       </c>
@@ -12326,7 +12440,7 @@
         <v>-1.21740165450427E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>8</v>
       </c>
@@ -12349,9 +12463,9 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F34"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
@@ -12361,7 +12475,7 @@
     <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -12375,7 +12489,7 @@
         <v>9.5583254269994297E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -12395,7 +12509,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0</v>
       </c>
@@ -12415,7 +12529,7 @@
         <v>2.27901221423021E-4</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -12435,7 +12549,7 @@
         <v>2.31108570802218E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2</v>
       </c>
@@ -12455,7 +12569,7 @@
         <v>2.55072751944751E-4</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>
@@ -12475,7 +12589,7 @@
         <v>1.33229755167912E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>4</v>
       </c>
@@ -12495,7 +12609,7 @@
         <v>-2.8956791023078102E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>5</v>
       </c>
@@ -12515,7 +12629,7 @@
         <v>1.55060996987099E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>6</v>
       </c>
@@ -12535,7 +12649,7 @@
         <v>1.3370711879616599E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>7</v>
       </c>
@@ -12555,7 +12669,7 @@
         <v>-2.64351000704543E-4</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>8</v>
       </c>
@@ -12575,7 +12689,7 @@
         <v>-1.7008091382262299E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>9</v>
       </c>
@@ -12595,7 +12709,7 @@
         <v>-4.7348999076028903E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10</v>
       </c>
@@ -12615,7 +12729,7 @@
         <v>-1.9583094439135001E-4</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>11</v>
       </c>
@@ -12635,7 +12749,7 @@
         <v>-1.01979899980586E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>12</v>
       </c>
@@ -12655,7 +12769,7 @@
         <v>-1.6976618436987301E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>13</v>
       </c>
@@ -12675,7 +12789,7 @@
         <v>1.3509037897166899E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>14</v>
       </c>
@@ -12695,7 +12809,7 @@
         <v>-4.0251692337766598E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>15</v>
       </c>
@@ -12715,7 +12829,7 @@
         <v>-3.9144852080597002E-3</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>16</v>
       </c>
@@ -12735,7 +12849,7 @@
         <v>-1.2018872661650401E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>17</v>
       </c>
@@ -12755,7 +12869,7 @@
         <v>6.9685420040077595E-4</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>18</v>
       </c>
@@ -12775,7 +12889,7 @@
         <v>8.8558447095388095E-4</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>19</v>
       </c>
@@ -12795,7 +12909,7 @@
         <v>3.3914477067993301E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>20</v>
       </c>
@@ -12815,7 +12929,7 @@
         <v>-3.6699534450201901E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>21</v>
       </c>
@@ -12835,7 +12949,7 @@
         <v>1.6901728547010701E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>22</v>
       </c>
@@ -12855,7 +12969,7 @@
         <v>3.5566008574485701E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>23</v>
       </c>
@@ -12875,7 +12989,7 @@
         <v>2.34240809806618E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>24</v>
       </c>
@@ -12895,7 +13009,7 @@
         <v>-3.8331853111473698E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>25</v>
       </c>
@@ -12915,7 +13029,7 @@
         <v>-4.2334451023048301E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>26</v>
       </c>
@@ -12935,7 +13049,7 @@
         <v>1.35265354365587E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>27</v>
       </c>
@@ -12955,7 +13069,7 @@
         <v>-2.94054514192437E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>28</v>
       </c>
@@ -12975,7 +13089,7 @@
         <v>-6.8809596209191597E-3</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>29</v>
       </c>
@@ -12995,7 +13109,7 @@
         <v>-5.1583751087591601E-4</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>8</v>
       </c>
@@ -13017,11 +13131,11 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:I27"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="2:9">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B2" s="8" t="s">
         <v>10</v>
       </c>
@@ -13035,7 +13149,7 @@
       </c>
       <c r="G2" s="14"/>
     </row>
-    <row r="3" spans="2:9">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
       <c r="D3" s="6" t="s">
@@ -13051,7 +13165,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="2:9">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="16" t="s">
         <v>11</v>
       </c>
@@ -13075,7 +13189,7 @@
         <v>7159.1722375171821</v>
       </c>
     </row>
-    <row r="5" spans="2:9">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="16"/>
       <c r="C5" s="9" t="s">
         <v>13</v>
@@ -13101,7 +13215,7 @@
         <v>5.2434513633378645E-4</v>
       </c>
     </row>
-    <row r="6" spans="2:9">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="16"/>
       <c r="C6" s="9" t="s">
         <v>14</v>
@@ -13127,7 +13241,7 @@
         <v>8.797703848114102E-3</v>
       </c>
     </row>
-    <row r="7" spans="2:9">
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="17"/>
       <c r="C7" s="10" t="s">
         <v>16</v>
@@ -13149,7 +13263,7 @@
         <v>3.6099371088204111E-3</v>
       </c>
     </row>
-    <row r="8" spans="2:9">
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" s="15" t="s">
         <v>18</v>
       </c>
@@ -13173,7 +13287,7 @@
         <v>11295.447664038575</v>
       </c>
     </row>
-    <row r="9" spans="2:9">
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B9" s="16"/>
       <c r="C9" s="9" t="s">
         <v>13</v>
@@ -13195,7 +13309,7 @@
         <v>1.4868639033140696E-2</v>
       </c>
     </row>
-    <row r="10" spans="2:9">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="16"/>
       <c r="C10" s="9" t="s">
         <v>14</v>
@@ -13217,7 +13331,7 @@
         <v>0.12172660266913846</v>
       </c>
     </row>
-    <row r="11" spans="2:9">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="17"/>
       <c r="C11" s="10" t="s">
         <v>16</v>
@@ -13239,7 +13353,7 @@
         <v>5.7688357787110244E-3</v>
       </c>
     </row>
-    <row r="12" spans="2:9">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="15" t="s">
         <v>20</v>
       </c>
@@ -13263,7 +13377,7 @@
         <v>9862.3957827047598</v>
       </c>
     </row>
-    <row r="13" spans="2:9">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="16"/>
       <c r="C13" s="9" t="s">
         <v>13</v>
@@ -13285,7 +13399,7 @@
         <v>1.4358361485530238E-2</v>
       </c>
     </row>
-    <row r="14" spans="2:9">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="16"/>
       <c r="C14" s="9" t="s">
         <v>14</v>
@@ -13307,7 +13421,7 @@
         <v>2.4086556702087061E-2</v>
       </c>
     </row>
-    <row r="15" spans="2:9">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B15" s="17"/>
       <c r="C15" s="10" t="s">
         <v>16</v>
@@ -13329,7 +13443,7 @@
         <v>2.7756297086266094E-2</v>
       </c>
     </row>
-    <row r="16" spans="2:9">
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B16" s="15" t="s">
         <v>19</v>
       </c>
@@ -13353,7 +13467,7 @@
         <v>11662.834674455355</v>
       </c>
     </row>
-    <row r="17" spans="2:7">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="16"/>
       <c r="C17" s="9" t="s">
         <v>13</v>
@@ -13375,7 +13489,7 @@
         <v>0.14256837030049149</v>
       </c>
     </row>
-    <row r="18" spans="2:7">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="16"/>
       <c r="C18" s="9" t="s">
         <v>14</v>
@@ -13397,7 +13511,7 @@
         <v>0.30035859770009959</v>
       </c>
     </row>
-    <row r="19" spans="2:7">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="17"/>
       <c r="C19" s="10" t="s">
         <v>16</v>
@@ -13419,7 +13533,7 @@
         <v>0.19898209936606981</v>
       </c>
     </row>
-    <row r="20" spans="2:7">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="15" t="s">
         <v>21</v>
       </c>
@@ -13443,7 +13557,7 @@
         <v>6152.0915049320811</v>
       </c>
     </row>
-    <row r="21" spans="2:7">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="16"/>
       <c r="C21" s="9" t="s">
         <v>13</v>
@@ -13465,7 +13579,7 @@
         <v>4.8120945537095663E-3</v>
       </c>
     </row>
-    <row r="22" spans="2:7">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="16"/>
       <c r="C22" s="9" t="s">
         <v>14</v>
@@ -13487,7 +13601,7 @@
         <v>1.1788804032500315E-2</v>
       </c>
     </row>
-    <row r="23" spans="2:7">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="17"/>
       <c r="C23" s="10" t="s">
         <v>16</v>
@@ -13509,7 +13623,7 @@
         <v>8.9307924910633947E-3</v>
       </c>
     </row>
-    <row r="24" spans="2:7">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="15" t="s">
         <v>23</v>
       </c>
@@ -13533,7 +13647,7 @@
         <v>8324.0242257182817</v>
       </c>
     </row>
-    <row r="25" spans="2:7">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" s="16"/>
       <c r="C25" s="9" t="s">
         <v>13</v>
@@ -13555,7 +13669,7 @@
         <v>1.1927708306011145E-3</v>
       </c>
     </row>
-    <row r="26" spans="2:7">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="16"/>
       <c r="C26" s="9" t="s">
         <v>14</v>
@@ -13577,7 +13691,7 @@
         <v>2.2290736833031916E-3</v>
       </c>
     </row>
-    <row r="27" spans="2:7">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B27" s="17"/>
       <c r="C27" s="10" t="s">
         <v>16</v>

</xml_diff>